<commit_message>
Add the retailer balance report, unwired Sub API, and module checklists.
Commission docs now follow % of sales, and Reports includes the client Retailer Credits ledger. The Sub API client stays unwired.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/esari-computations.xlsx
+++ b/docs/esari-computations.xlsx
@@ -536,7 +536,7 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commission pool / sale margin</t>
+          <t xml:space="preserve">Sale Margin (leftover after credits)</t>
         </is>
       </c>
       <c r="B8" s="8">
@@ -544,14 +544,14 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The remaining 3%. This is the pool, not one party’s profit</t>
+          <t xml:space="preserve">Inventory leftover. Not the commission base.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commission split (Retailer A demo defaults)</t>
+          <t xml:space="preserve">Commission split — % of sales (demo defaults 10 / 20 / 30 / 40)</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B11" s="10">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="12">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B13" s="10">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="14">
@@ -613,7 +613,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Share of pool (₱)</t>
+          <t xml:space="preserve">Share of sales (₱)</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="B18" s="8">
-        <f>ROUND($B$8*B11,2)</f>
+        <f>ROUND($B$2*B11,2)</f>
       </c>
     </row>
     <row r="19">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="B19" s="8">
-        <f>ROUND($B$8*B12,2)</f>
+        <f>ROUND($B$2*B12,2)</f>
       </c>
     </row>
     <row r="20">
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B20" s="8">
-        <f>ROUND($B$8*B13,2)</f>
+        <f>ROUND($B$2*B13,2)</f>
       </c>
     </row>
     <row r="21">
@@ -659,11 +659,11 @@
         </is>
       </c>
       <c r="B21" s="8">
-        <f>ROUND($B$8-B18-B19-B20,2)</f>
+        <f>ROUND($B$2-B18-B19-B20,2)</f>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not ROUND(pool×40%) — leftover cents go here</t>
+          <t xml:space="preserve">Not ROUND(sales×40%) — leftover cents go here</t>
         </is>
       </c>
     </row>
@@ -678,14 +678,14 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Must equal the commission pool</t>
+          <t xml:space="preserve">Must equal the customer payment</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sub-Franchisee remainder % (how Commission Settings fills SF)</t>
+          <t xml:space="preserve">Sub-Franchisee remainder % (Admin dialog)</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B25" s="10">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="26">
@@ -712,7 +712,7 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platform share % (fixed when a Sub exists)</t>
+          <t xml:space="preserve">Platform share % (Admin-set)</t>
         </is>
       </c>
       <c r="B27" s="10">
@@ -730,14 +730,14 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SF% = 100% − retailer − franchisee − platform</t>
+          <t xml:space="preserve">Admin: SF% = 100% − retailer − franchisee − platform</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retailer B demo plan: 30% / 15% / 15% / 40%. New Commission Settings dialog defaults: 30% / 20% / 10% / 40%.</t>
+          <t xml:space="preserve">Sub-Franchisee dialog: retailer, franchisee, and Your Share are editable; platform fee is read-only. Four % must equal 100% of sales. Demo seed for every retailer: 10% / 20% / 30% / 40%.</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5. ₱1,000 Retailer A demo sale (25 / 20 / 15 / 40)</t>
+          <t xml:space="preserve">5. ₱1,000 Retailer A demo sale (10 / 20 / 30 / 40 of sales)</t>
         </is>
       </c>
     </row>
@@ -1036,14 +1036,14 @@
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97% of ₱1,000 = ₱970</t>
+          <t xml:space="preserve">97% of ₱1,000 = ₱970 (inventory)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commission pool</t>
+          <t xml:space="preserve">Sale Margin (leftover after credits)</t>
         </is>
       </c>
       <c r="B32" s="8">
@@ -1051,52 +1051,52 @@
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1,000 − 970 = 30</t>
+          <t xml:space="preserve">1,000 − 970 = 30 — not the commission base</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retailer A 25%</t>
+          <t xml:space="preserve">Retailer A 10% of sales</t>
         </is>
       </c>
       <c r="B33" s="8">
-        <f>ROUND(B32*0.25,2)</f>
+        <f>ROUND(B30*0.10,2)</f>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.50</t>
+          <t xml:space="preserve">100.00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Franchisee A 20%</t>
+          <t xml:space="preserve">Franchisee A 20% of sales</t>
         </is>
       </c>
       <c r="B34" s="8">
-        <f>ROUND(B32*0.20,2)</f>
+        <f>ROUND(B30*0.20,2)</f>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.00</t>
+          <t xml:space="preserve">200.00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sub-Franchisee 15%</t>
+          <t xml:space="preserve">Sub-Franchisee 30% of sales</t>
         </is>
       </c>
       <c r="B35" s="8">
-        <f>ROUND(B32*0.15,2)</f>
+        <f>ROUND(B30*0.30,2)</f>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.50</t>
+          <t xml:space="preserve">300.00</t>
         </is>
       </c>
     </row>
@@ -1107,11 +1107,11 @@
         </is>
       </c>
       <c r="B36" s="8">
-        <f>ROUND(B32-B33-B34-B35,2)</f>
+        <f>ROUND(B30-B33-B34-B35,2)</f>
       </c>
       <c r="D36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">12.00</t>
+          <t xml:space="preserve">400.00</t>
         </is>
       </c>
     </row>
@@ -1329,20 +1329,20 @@
         </is>
       </c>
       <c r="B11" s="9">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="C11" s="9">
         <v>0.2</v>
       </c>
       <c r="D11" s="9">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="E11" s="9">
         <v>0.4</v>
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">sharePlans[0]; SF is remainder</t>
+          <t xml:space="preserve">% of sales; demo seed</t>
         </is>
       </c>
     </row>
@@ -1353,20 +1353,20 @@
         </is>
       </c>
       <c r="B12" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="C12" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="D12" s="9">
         <v>0.3</v>
-      </c>
-      <c r="C12" s="9">
-        <v>0.15</v>
-      </c>
-      <c r="D12" s="9">
-        <v>0.15</v>
       </c>
       <c r="E12" s="9">
         <v>0.4</v>
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">sharePlans[1]; SF is remainder</t>
+          <t xml:space="preserve">Same default as A</t>
         </is>
       </c>
     </row>
@@ -1377,20 +1377,20 @@
         </is>
       </c>
       <c r="B13" s="9">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="C13" s="9">
         <v>0.2</v>
       </c>
       <c r="D13" s="9">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="E13" s="9">
         <v>0.4</v>
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same plan as A (index 2 % 2)</t>
+          <t xml:space="preserve">Same default as A</t>
         </is>
       </c>
     </row>
@@ -1401,20 +1401,20 @@
         </is>
       </c>
       <c r="B14" s="9">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="C14" s="9">
         <v>0.2</v>
       </c>
       <c r="D14" s="9">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E14" s="9">
         <v>0.4</v>
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEFAULT_SHARE_PERCENTAGES if you create a new row</t>
+          <t xml:space="preserve">DEFAULT_SHARE_PERCENTAGES</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sum of your stamped % × pool on completed sales in the period</t>
+          <t xml:space="preserve">Sum of your stamped % of sales on completed sales in the period</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">This workbook is the same math the demo app uses (18 August 2026). Grey cells are formulas — do not type over them. Excel recalculates on open. Open the Load calculator or Sale calculator tabs to edit yellow inputs.</t>
+          <t xml:space="preserve">This workbook is the same math the demo app uses (1 September 2026). Grey cells are formulas — do not type over them. Excel recalculates on open. Open the Load calculator or Sale calculator tabs to edit yellow inputs.</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your % of the commission pool (customer payment − credits consumed)</t>
+          <t xml:space="preserve">Your % of the customer payment (Sales)</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo sale: 97% credits consumed, then the 4-tier commission split</t>
+          <t xml:space="preserve">Demo sale: 97% credits consumed (inventory); Commission Settings % of sales</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Numbers used in the user guide (₱30,000 load, ₱1,000 sale, Retailer A split)</t>
+          <t xml:space="preserve">Numbers used in the user guide (₱30,000 load, ₱1,000 sale, 10 / 20 / 30 / 40 of sales)</t>
         </is>
       </c>
     </row>
@@ -1948,12 +1948,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commission pool / sale margin</t>
+          <t xml:space="preserve">Sale Margin (leftover after credits)</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">pool = customer_payment − credits_consumed</t>
+          <t xml:space="preserve">leftover = customer_payment − credits_consumed</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transactions, Transaction Details, Wallet Sale Margin</t>
+          <t xml:space="preserve">Transactions, Transaction Details, Wallet Sale Margin — not the commission base</t>
         </is>
       </c>
     </row>
@@ -1975,12 +1975,12 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">share = pool × party_% ÷ 100</t>
+          <t xml:space="preserve">share = customer_payment × party_% ÷ 100</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROUND(pool*pct/100,2)</t>
+          <t xml:space="preserve">ROUND(payment*pct/100,2)</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -1997,12 +1997,12 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">platform = pool − retailer − franchisee − sub-franchisee</t>
+          <t xml:space="preserve">platform = payment − retailer − franchisee − sub-franchisee</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROUND(pool-ret-fran-sub,2)</t>
+          <t xml:space="preserve">ROUND(payment-ret-fran-sub,2)</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
@@ -2014,7 +2014,7 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sub-Franchisee remainder %</t>
+          <t xml:space="preserve">Sub-Franchisee remainder % (Admin dialog)</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commission Settings when a Sub-Franchisee exists</t>
+          <t xml:space="preserve">Admin Commission Settings — Sub share is remainder; platform fee is Admin-editable</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Burn 100% of sales from Available Credits and hide Sale Margin.
The 2% processing-fee haircut is gone, so a ₱1,000 sale now debits ₱1,000 of inventory.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/esari-computations.xlsx
+++ b/docs/esari-computations.xlsx
@@ -525,26 +525,11 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>ROUND(B2*0.97,2)</f>
+        <f>B2</f>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97% of payment — burned from Available Credits</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sale Margin (leftover after credits)</t>
-        </is>
-      </c>
-      <c r="B8" s="8">
-        <f>ROUND(B6-B7,2)</f>
-      </c>
-      <c r="C8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inventory leftover. Not the commission base.</t>
+          <t xml:space="preserve">100% of payment — burned from Available Credits</t>
         </is>
       </c>
     </row>
@@ -1032,26 +1017,11 @@
         </is>
       </c>
       <c r="B31" s="8">
-        <f>ROUND(B30*0.97,2)</f>
+        <f>B30</f>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97% of ₱1,000 = ₱970 (inventory)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sale Margin (leftover after credits)</t>
-        </is>
-      </c>
-      <c r="B32" s="8">
-        <f>ROUND(B30-B31,2)</f>
-      </c>
-      <c r="D32" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1,000 − 970 = 30 — not the commission base</t>
+          <t xml:space="preserve">100% of ₱1,000 = ₱1,000 (inventory)</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1123,7 @@
       </c>
       <c r="D41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6,250 − 970 = 5,280  (Sufficient, above ₱5,000)</t>
+          <t xml:space="preserve">6,250 − 1,000 = 5,250  (Sufficient, above ₱5,000)</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1709,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Demo sale: 97% credits consumed (inventory); Commission Settings % of sales</t>
+          <t xml:space="preserve">Demo sale: 100% credits consumed (inventory); Commission Settings % of sales</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1767,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1931,12 +1901,12 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">credits_consumed = customer_payment × 97%</t>
+          <t xml:space="preserve">credits_consumed = customer_payment</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROUND(payment*0.97,2)</t>
+          <t xml:space="preserve">ROUND(payment,2)</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
@@ -1948,203 +1918,181 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sale Margin (leftover after credits)</t>
+          <t xml:space="preserve">Party commission</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">leftover = customer_payment − credits_consumed</t>
+          <t xml:space="preserve">share = customer_payment × party_% ÷ 100</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROUND(payment-credits_consumed,2)</t>
+          <t xml:space="preserve">ROUND(payment*pct/100,2)</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transactions, Transaction Details, Wallet Sale Margin — not the commission base</t>
+          <t xml:space="preserve">Transaction Details, Revenue Sales Commission, Reports</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Party commission</t>
+          <t xml:space="preserve">Platform remainder</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">share = customer_payment × party_% ÷ 100</t>
+          <t xml:space="preserve">platform = payment − retailer − franchisee − sub-franchisee</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROUND(payment*pct/100,2)</t>
+          <t xml:space="preserve">ROUND(payment-ret-fran-sub,2)</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transaction Details, Revenue Sales Commission, Reports</t>
+          <t xml:space="preserve">Transaction Details (absorbs 1-cent rounding)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platform remainder</t>
+          <t xml:space="preserve">Sub-Franchisee remainder % (Admin dialog)</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">platform = payment − retailer − franchisee − sub-franchisee</t>
+          <t xml:space="preserve">SF% = max(0, 100 − retailer% − franchisee% − platform%)</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROUND(payment-ret-fran-sub,2)</t>
+          <t xml:space="preserve">MAX(0,1-ret-fran-plat)</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transaction Details (absorbs 1-cent rounding)</t>
+          <t xml:space="preserve">Admin Commission Settings — Sub share is remainder; platform fee is Admin-editable</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sub-Franchisee remainder % (Admin dialog)</t>
+          <t xml:space="preserve">Total earnings (Sub/Fran)</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SF% = max(0, 100 − retailer% − franchisee% − platform%)</t>
+          <t xml:space="preserve">total = IC earnings + Sales Commission (credited)</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAX(0,1-ret-fran-plat)</t>
+          <t xml:space="preserve">ic_earnings+sales_commission</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admin Commission Settings — Sub share is remainder; platform fee is Admin-editable</t>
+          <t xml:space="preserve">Revenue hero cards</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total earnings (Sub/Fran)</t>
+          <t xml:space="preserve">Available Credits</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">total = IC earnings + Sales Commission (credited)</t>
+          <t xml:space="preserve">available = opening + received − released − consumed on sales</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ic_earnings+sales_commission</t>
+          <t xml:space="preserve">opening+in-out-consumed</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revenue hero cards</t>
+          <t xml:space="preserve">Wallets / Wallet, after-release preview</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Available Credits</t>
+          <t xml:space="preserve">Low Balance</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">available = opening + received − released − consumed on sales</t>
+          <t xml:space="preserve">0 &lt; available ≤ 5,000</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">opening+in-out-consumed</t>
+          <t xml:space="preserve">AND(available&gt;0,available&lt;=5000)</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wallets / Wallet, after-release preview</t>
+          <t xml:space="preserve">Wallet banner, bell, status badge</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low Balance</t>
+          <t xml:space="preserve">Zero Balance</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 &lt; available ≤ 5,000</t>
+          <t xml:space="preserve">available ≤ 0</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">AND(available&gt;0,available&lt;=5000)</t>
+          <t xml:space="preserve">available&lt;=0</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wallet banner, bell, status badge</t>
+          <t xml:space="preserve">Wallet banner (red), bell</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zero Balance</t>
+          <t xml:space="preserve">Sufficient</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">available ≤ 0</t>
+          <t xml:space="preserve">available &gt; 5,000</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">available&lt;=0</t>
+          <t xml:space="preserve">available&gt;5000</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wallet banner (red), bell</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sufficient</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">available &gt; 5,000</t>
-        </is>
-      </c>
-      <c r="C16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">available&gt;5000</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
           <t xml:space="preserve">Wallet status badge</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Do not use “deposit + %”. Credits are always deposit divided by the rate.</t>
         </is>

</xml_diff>